<commit_message>
depin: Commission Factory contact judgment and first note
Name-free record: company facts (Awin full acquisition 2020, MY/SG
offices), advertiser-side public titles to approach, 295-char note,
prerequisites. Contacts xlsx row 6 updated. Also logs the merged
Wellbian Cafe quote.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014drgzQYBXTLjd1zzmsjRaS
</commit_message>
<xml_diff>
--- a/depin/content/affiliate-contacts-1019.xlsx
+++ b/depin/content/affiliate-contacts-1019.xlsx
@@ -1230,7 +1230,84 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">호주</t>
+      <t xml:space="preserve">호주 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">뉴질랜드 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동남아</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(CF </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">말레이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">싱가포르 사무소</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -1257,7 +1334,84 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">대형 퍼블리셔 풀</t>
+      <t xml:space="preserve">대형 퍼블리셔 풀 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· CF = 2011 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">호주 설립</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, Awin 2020.9 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전량 인수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">브랜드 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">600+(2020 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자체</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -1293,37 +1447,207 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(CE/RED)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">New Business — APAC / EU</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">유럽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">호주 배송 정한 뒤</t>
+      <t xml:space="preserve">(CE/RED) · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">호주 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">뉴질랜드 배송 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기기 인증</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(RCM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">여부 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Enterprise Commercial · Strategic Partnerships(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">광고주 쪽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CF </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">광고주 쪽 공개 직함 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">촌 메모</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10/20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초안 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">295</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) — vCommission </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메일 뒤</t>
     </r>
   </si>
   <si>
@@ -5794,7 +6118,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
@@ -5819,7 +6143,7 @@
       <c r="H10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="I10" s="5" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
depin: Involve Asia contact judgment and first note
Name-free record: who in the search results actually works there,
which advertiser-side title to approach, 297-char note, and the public
self-serve advertiser sign-up as a fallback. Contacts xlsx row 2 updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014drgzQYBXTLjd1zzmsjRaS
</commit_message>
<xml_diff>
--- a/depin/content/affiliate-contacts-1019.xlsx
+++ b/depin/content/affiliate-contacts-1019.xlsx
@@ -489,13 +489,206 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">동남아 배송 국가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Head of Partnerships · Advertiser BD · Country Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">링크드인 직함 찾기</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동남아 배송 국가 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">크립토 연관 광고주 심사 미확인</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Partner Growth · Business Development(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">광고주 쪽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BD </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">겸 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Partner Growth </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시니어 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">촌 메모</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10/20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초안 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">297</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일주일 무응답이면 공식 광고주 가입 양식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">셀프 가입 있음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">vCommission</t>
@@ -6002,7 +6195,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
@@ -6027,7 +6220,7 @@
       <c r="H6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="5" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
depin: ACCESSTRADE contact judgment and first note
Name-free record: global business director as the Southeast Asia
entry point, Japan lane held until radio certification, 298-char note,
and a note on keeping answers consistent across the four networks.
Contacts xlsx row 5 updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014drgzQYBXTLjd1zzmsjRaS
</commit_message>
<xml_diff>
--- a/depin/content/affiliate-contacts-1019.xlsx
+++ b/depin/content/affiliate-contacts-1019.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="213">
   <si>
     <r>
       <rPr>
@@ -1317,7 +1317,101 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">일본 확장 때 그대로</t>
+      <t xml:space="preserve">일본 확장 때 그대로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· Interspace(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일본</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">운영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">베트남은 합작 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· 6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개국</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자체</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -1370,618 +1464,780 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Global BD · Advertiser Sales</t>
+      <t xml:space="preserve">0 · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동남아는 배송 국가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Director of Global Business(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">호치민</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동남아 먼저 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Global Business </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">디렉터 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명에 메모</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10/20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초안 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">298</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일본 쪽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도쿄 미디어 세일즈</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 인증 뒤</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Awin · Commission Factory(APAC)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유럽 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미국 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">호주 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">뉴질랜드 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">동남아</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(CF </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">말레이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">싱가포르 사무소</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실물 상품 광고주에 강함 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대형 퍼블리셔 풀 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· CF = 2011 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">호주 설립</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, Awin 2020.9 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전량 인수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">브랜드 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">600+(2020 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자체</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">크립토 연관 심사 보수적일 가능성 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유럽 기기 인증</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(CE/RED) · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">호주 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">뉴질랜드 배송 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기기 인증</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(RCM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">여부 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Enterprise Commercial · Strategic Partnerships(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">광고주 쪽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CF </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">광고주 쪽 공개 직함 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">촌 메모</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10/20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초안 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">295</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) — vCommission </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메일 뒤</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">A8.net · ValueCommerce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">일본</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">광고주 대시보드 영문 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">광고주 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자체</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) · ValueCommerce </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">해외 광고주 일본 진출 이력</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일본 법인 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">세무 요건 미확인 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전파법 인증</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Global / Overseas Sales</t>
   </si>
   <si>
     <t xml:space="preserve">일본 인증 상태 확인 뒤</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Awin · Commission Factory(APAC)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">유럽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">미국 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">호주 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">뉴질랜드 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">동남아</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(CF </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">말레이 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">싱가포르 사무소</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">실물 상품 광고주에 강함 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">대형 퍼블리셔 풀 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· CF = 2011 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">호주 설립</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, Awin 2020.9 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">전량 인수</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">브랜드 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">600+(2020 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">자체</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">크립토 연관 심사 보수적일 가능성 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">유럽 기기 인증</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(CE/RED) · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">호주 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">뉴질랜드 배송 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">기기 인증</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(RCM </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">여부 확인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Enterprise Commercial · Strategic Partnerships(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">광고주 쪽</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">CF </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">광고주 쪽 공개 직함 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">명에 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">촌 메모</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(10/20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">초안 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">295</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">자</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) — vCommission </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">메일 뒤</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">A8.net · ValueCommerce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">일본</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">A8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">광고주 대시보드 영문 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">광고주 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2.7</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">만</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">자체</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) · ValueCommerce </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">해외 광고주 일본 진출 이력</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일본 법인 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">세무 요건 미확인 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">전파법 인증</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Global / Overseas Sales</t>
   </si>
   <si>
     <t xml:space="preserve">Admitad</t>
@@ -6282,7 +6538,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
@@ -6366,7 +6622,7 @@
         <v>17</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6374,28 +6630,28 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>17</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6403,28 +6659,28 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>17</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6432,28 +6688,28 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>17</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6461,28 +6717,28 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>17</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6490,28 +6746,28 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6519,28 +6775,28 @@
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>17</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6548,28 +6804,28 @@
         <v>14</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>17</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -6611,29 +6867,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>9</v>
@@ -6642,111 +6898,111 @@
         <v>10</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>31</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -6785,229 +7041,229 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -7045,96 +7301,96 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>196</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -7164,7 +7420,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7175,10 +7431,10 @@
         <v>21</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7200,7 +7456,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B5" s="12" t="n">
         <f aca="false">COUNTIF(네트워크!$H$5:$H$18,$A5)</f>
@@ -7234,7 +7490,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">COUNTIF(네트워크!$H$5:$H$18,$A7)</f>
@@ -7251,7 +7507,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">COUNTIF(네트워크!$H$5:$H$18,$A8)</f>
@@ -7268,7 +7524,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">COUNTIF(네트워크!$H$5:$H$18,$A9)</f>
@@ -7285,7 +7541,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">COUNTIF(네트워크!$H$5:$H$18,$A10)</f>
@@ -7302,7 +7558,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">COUNTIF(네트워크!$H$5:$H$18,$A11)</f>
@@ -7319,7 +7575,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B12" s="13" t="n">
         <f aca="false">SUM(B4:B11)</f>
@@ -7336,7 +7592,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
depin: vCommission advertiser team looped in; follow-up drafted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014drgzQYBXTLjd1zzmsjRaS
</commit_message>
<xml_diff>
--- a/depin/content/affiliate-contacts-1019.xlsx
+++ b/depin/content/affiliate-contacts-1019.xlsx
@@ -933,58 +933,100 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Disha </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">메일 주소 받으면 광고주 정보 메일 발송</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">질문 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">포함</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
+      <t xml:space="preserve">10/19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메일 발송 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">같은 날 광고주 팀 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명 연결 → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10/20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통화 요청</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10/24 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보상 「테스트」 문구 정정</t>
     </r>
   </si>
   <si>
@@ -6480,7 +6522,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
depin: vCommission follow-up by email only, no call
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014drgzQYBXTLjd1zzmsjRaS
</commit_message>
<xml_diff>
--- a/depin/content/affiliate-contacts-1019.xlsx
+++ b/depin/content/affiliate-contacts-1019.xlsx
@@ -992,33 +992,33 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">통화 요청</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(10/24 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">전</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) · </t>
+      <t xml:space="preserve">서면 질의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통화 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">X) · </t>
     </r>
     <r>
       <rPr>

</xml_diff>